<commit_message>
refactor: set test environment, handle kwargs argument. feat: implemented logger, implemented entry point to backend logic
</commit_message>
<xml_diff>
--- a/app/tests/clients_export.xlsx
+++ b/app/tests/clients_export.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,7 +444,17 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>display_name</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>created_at</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>updated_at</t>
         </is>
       </c>
     </row>
@@ -476,7 +486,17 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2025-11-03 14:14:46</t>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-03-19 10:02:23</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-03-19 10:02:23</t>
         </is>
       </c>
     </row>
@@ -508,7 +528,17 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2025-11-03 14:14:46</t>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-03-19 10:02:23</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-03-19 10:02:23</t>
         </is>
       </c>
     </row>
@@ -540,7 +570,17 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2025-11-03 14:14:47</t>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-03-19 10:02:23</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-03-19 10:02:23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement dynamic argument processing with validation for entry point
</commit_message>
<xml_diff>
--- a/app/tests/clients_export.xlsx
+++ b/app/tests/clients_export.xlsx
@@ -491,12 +491,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-03-19 10:02:23</t>
+          <t>2026-03-19 16:23:55</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-03-19 10:02:23</t>
+          <t>2026-03-19 16:23:55</t>
         </is>
       </c>
     </row>
@@ -533,12 +533,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-03-19 10:02:23</t>
+          <t>2026-03-19 16:23:55</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-03-19 10:02:23</t>
+          <t>2026-03-19 16:23:55</t>
         </is>
       </c>
     </row>
@@ -575,12 +575,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-03-19 10:02:23</t>
+          <t>2026-03-19 16:23:55</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-03-19 10:02:23</t>
+          <t>2026-03-19 16:23:55</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement tablemap for dynamic db query accross models
</commit_message>
<xml_diff>
--- a/app/tests/clients_export.xlsx
+++ b/app/tests/clients_export.xlsx
@@ -413,46 +413,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>first_name</t>
+          <t>plan_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>last_name</t>
+          <t>client_id</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>company_name</t>
+          <t>plan_unit</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>expiration_date</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>phone</t>
+          <t>discount</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>display_name</t>
+          <t>discount_type</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>vat</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>payment_status</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>updated_at</t>
         </is>
@@ -461,126 +476,51 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Client</t>
+          <t>e170a7b4-04ab-405b-9101-9963fa30ac03</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Two</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Two Company</t>
-        </is>
+          <t>12b47c8d-cd87-44bf-b4dc-72962d061c6f</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>2</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>clienttwo@mail.com</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>081000000002</t>
-        </is>
+          <t>2026-03-23 10:06:57</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>0.1</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>client</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2026-03-19 16:23:55</t>
-        </is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>0.1</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-03-19 16:23:55</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Client</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Three</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Three Company</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>clientthree@mail.com</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>081000000003</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>client</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2026-03-19 16:23:55</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>2026-03-19 16:23:55</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Client</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Four</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Four Company</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>clientfour@mail.com</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>081000000004</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>client</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2026-03-19 16:23:55</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>2026-03-19 16:23:55</t>
+          <t>booked</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2026-03-21 10:06:57</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2026-03-21 10:06:57</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: dynamically create db tables using TABLE_MAP
</commit_message>
<xml_diff>
--- a/app/tests/clients_export.xlsx
+++ b/app/tests/clients_export.xlsx
@@ -476,12 +476,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>e170a7b4-04ab-405b-9101-9963fa30ac03</t>
+          <t>46ac6009-d282-4d8f-932f-f12d1dccc4e8</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>12b47c8d-cd87-44bf-b4dc-72962d061c6f</t>
+          <t>efcc1be7-afe0-43c0-9795-454da440fe19</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -489,7 +489,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-23 10:06:57</t>
+          <t>2026-03-24 08:16:35</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -515,12 +515,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-03-21 10:06:57</t>
+          <t>2026-03-22 08:16:35</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-03-21 10:06:57</t>
+          <t>2026-03-22 08:16:35</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
doc: code documentation and cleanup
</commit_message>
<xml_diff>
--- a/app/tests/clients_export.xlsx
+++ b/app/tests/clients_export.xlsx
@@ -476,12 +476,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>46ac6009-d282-4d8f-932f-f12d1dccc4e8</t>
+          <t>efc7abf3-754b-4bb7-a9a9-c2d964d6cdc1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>efcc1be7-afe0-43c0-9795-454da440fe19</t>
+          <t>1e67dc50-57c1-4a88-9241-436f1ed5ca16</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -489,7 +489,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-24 08:16:35</t>
+          <t>2026-03-24 10:38:46</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -515,12 +515,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-03-22 08:16:35</t>
+          <t>2026-03-22 10:38:46</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-03-22 08:16:35</t>
+          <t>2026-03-22 10:38:46</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: allow models to raise exceptions
</commit_message>
<xml_diff>
--- a/app/tests/clients_export.xlsx
+++ b/app/tests/clients_export.xlsx
@@ -476,12 +476,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>efc7abf3-754b-4bb7-a9a9-c2d964d6cdc1</t>
+          <t>4758a051-009a-45e8-bad5-e0150e0fac91</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1e67dc50-57c1-4a88-9241-436f1ed5ca16</t>
+          <t>a3ddad3e-09df-4a6b-b06b-aa7ecd0477de</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -489,7 +489,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-24 10:38:46</t>
+          <t>2026-03-24 13:51:21</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -515,12 +515,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-03-22 10:38:46</t>
+          <t>2026-03-22 13:51:21</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-03-22 10:38:46</t>
+          <t>2026-03-22 13:51:21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: made fk table created first
</commit_message>
<xml_diff>
--- a/app/tests/clients_export.xlsx
+++ b/app/tests/clients_export.xlsx
@@ -476,12 +476,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>4758a051-009a-45e8-bad5-e0150e0fac91</t>
+          <t>f29a166f-d63d-49a2-8ba8-93ff8eb2e9b6</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>a3ddad3e-09df-4a6b-b06b-aa7ecd0477de</t>
+          <t>3c35fcae-5f23-478d-88c5-312f378a7f58</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -489,7 +489,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-24 13:51:21</t>
+          <t>2026-04-30 07:48:07</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -515,12 +515,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-03-22 13:51:21</t>
+          <t>2026-04-28 07:48:07</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-03-22 13:51:21</t>
+          <t>2026-04-28 07:48:07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat:implement dyname table creation and model generation via command line
</commit_message>
<xml_diff>
--- a/app/tests/clients_export.xlsx
+++ b/app/tests/clients_export.xlsx
@@ -476,12 +476,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>f29a166f-d63d-49a2-8ba8-93ff8eb2e9b6</t>
+          <t>013cca99-c5e2-4fd1-bf06-4da0eb6f6345</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>3c35fcae-5f23-478d-88c5-312f378a7f58</t>
+          <t>0977a02a-ff63-47e5-a882-1f938c8b6367</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -489,7 +489,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-04-30 07:48:07</t>
+          <t>2026-04-30 20:05:25</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -515,12 +515,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-04-28 07:48:07</t>
+          <t>2026-04-28 20:05:25</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-04-28 07:48:07</t>
+          <t>2026-04-28 20:05:25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement direct model retrieval and creation, implement field instances
</commit_message>
<xml_diff>
--- a/app/tests/clients_export.xlsx
+++ b/app/tests/clients_export.xlsx
@@ -476,12 +476,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>46d54c0c-7baa-4e60-9e16-918a9c6e45fb</t>
+          <t>263e23bf-9a80-4c53-b528-9da44a016dec</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>c137944b-b942-4ff6-8068-87ebb326e92e</t>
+          <t>8c53c87b-2e56-47f2-b715-21cf082285a1</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -489,7 +489,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-04-30 21:09:45</t>
+          <t>2026-05-01 08:50:59</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -515,12 +515,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-04-28 21:09:45</t>
+          <t>2026-04-29 08:50:59</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-04-28 21:09:45</t>
+          <t>2026-04-29 08:50:59</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement fk field data handling with integrated test
</commit_message>
<xml_diff>
--- a/app/tests/clients_export.xlsx
+++ b/app/tests/clients_export.xlsx
@@ -434,22 +434,22 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>discount</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>discount_type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>vat</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>expiration_date</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>discount</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>discount_type</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>vat</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
@@ -476,32 +476,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>263e23bf-9a80-4c53-b528-9da44a016dec</t>
+          <t>ff671212-85c1-4351-8149-27f85f9b2463</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>8c53c87b-2e56-47f2-b715-21cf082285a1</t>
+          <t>79737ea3-9a96-4fbf-bec5-3f65e5888c6a</t>
         </is>
       </c>
       <c r="C2" t="n">
         <v>2</v>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-05-01 08:50:59</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F2" t="inlineStr">
+      <c r="D2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>percent</t>
         </is>
       </c>
-      <c r="G2" t="n">
-        <v>0.1</v>
+      <c r="F2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-05-03 20:23:14</t>
+        </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -515,12 +515,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-04-29 08:50:59</t>
+          <t>2026-05-03 20:23:14</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-04-29 08:50:59</t>
+          <t>2026-05-03 20:23:14</t>
         </is>
       </c>
     </row>

</xml_diff>